<commit_message>
Cambios Solicitados terminados 13-10-2020
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/ConsumoAgua/FORMATO REPORTE DE CONSUMO DE AGUA.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/ConsumoAgua/FORMATO REPORTE DE CONSUMO DE AGUA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Segunda Etapa\ConsumoAgua\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\ConsumoAgua\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{003A5B7E-8AB7-4480-9F07-C67005391E93}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0CE29C4-719A-497F-B671-6D7A2FC53E50}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{AFFB72D5-6F10-40F3-BC87-67601F9B819B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{AFFB72D5-6F10-40F3-BC87-67601F9B819B}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORTE MENSUAL" sheetId="1" r:id="rId1"/>
@@ -616,32 +616,32 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1360,28 +1360,28 @@
   </cols>
   <sheetData>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="14" t="s">
+      <c r="A6" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="14" t="s">
+      <c r="A7" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -1390,12 +1390,12 @@
       <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -1404,10 +1404,10 @@
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -1416,10 +1416,10 @@
       <c r="B11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -1428,10 +1428,10 @@
       <c r="B12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -1440,10 +1440,10 @@
       <c r="B13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -1452,10 +1452,10 @@
       <c r="B14" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -1464,10 +1464,10 @@
       <c r="B15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -1476,16 +1476,16 @@
       <c r="B16" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
     </row>
     <row r="18" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A18" s="18" t="s">
+      <c r="A18" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="19"/>
+      <c r="B18" s="17"/>
       <c r="C18" s="3" t="s">
         <v>13</v>
       </c>
@@ -1500,128 +1500,128 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="13" t="s">
+      <c r="A19" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="13"/>
+      <c r="B19" s="11"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="13" t="s">
+      <c r="A20" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="13"/>
+      <c r="B20" s="11"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="13" t="s">
+      <c r="A21" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="13"/>
+      <c r="B21" s="11"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="13"/>
+      <c r="B22" s="11"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="13" t="s">
+      <c r="A23" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="13"/>
+      <c r="B23" s="11"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="13" t="s">
+      <c r="A24" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="13"/>
+      <c r="B24" s="11"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="13" t="s">
+      <c r="A25" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="11"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="13" t="s">
+      <c r="A26" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="13"/>
+      <c r="B26" s="11"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="13" t="s">
+      <c r="A27" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="13"/>
+      <c r="B27" s="11"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="13" t="s">
+      <c r="A28" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="13"/>
+      <c r="B28" s="11"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="13" t="s">
+      <c r="A29" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="13"/>
+      <c r="B29" s="11"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="13" t="s">
+      <c r="A30" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="13"/>
+      <c r="B30" s="11"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="11"/>
-      <c r="B31" s="12"/>
+      <c r="A31" s="18"/>
+      <c r="B31" s="19"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
@@ -1629,6 +1629,18 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:F7"/>
@@ -1642,18 +1654,6 @@
     <mergeCell ref="C16:F16"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Mejoras consumo de agua
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/ConsumoAgua/FORMATO REPORTE DE CONSUMO DE AGUA.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/ConsumoAgua/FORMATO REPORTE DE CONSUMO DE AGUA.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\EData\Marcobre\Segunda Etapa\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\ConsumoAgua\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Segunda Etapa\ConsumoAgua\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\ConsumoAgua\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53D0A027-F1B5-4222-928C-75FD7B899327}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C18F562-758A-45ED-9E8A-483A196678AC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{AFFB72D5-6F10-40F3-BC87-67601F9B819B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{AFFB72D5-6F10-40F3-BC87-67601F9B819B}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORTE MENSUAL" sheetId="1" r:id="rId1"/>
     <sheet name="REPORTE CONSUMO DIARIO" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcOnSave="0" concurrentCalc="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -221,39 +221,7 @@
     <t>Tiempo de Bombeo (H)</t>
   </si>
   <si>
-    <t>Volumen de Agua Bombeado (consumo)
-m3</t>
-  </si>
-  <si>
     <t>Caudal promedio consumido (m3/s)</t>
-  </si>
-  <si>
-    <r>
-      <t>Lectura Inicial Flujometro en el día (m</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <vertAlign val="superscript"/>
-        <sz val="10"/>
-        <color theme="0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>3</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="0"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
   </si>
   <si>
     <r>
@@ -285,6 +253,37 @@
   </si>
   <si>
     <t>FORMATO DE REPORTE DE CONSUMO DE AGUA</t>
+  </si>
+  <si>
+    <r>
+      <t>Lectura Inicial Flujómetro en el día (m</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <vertAlign val="superscript"/>
+        <sz val="10"/>
+        <color theme="0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="0"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
+    <t>Volumen de Agua Bombeado (m3)</t>
   </si>
 </sst>
 </file>
@@ -616,32 +615,32 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1350,142 +1349,142 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51A04389-D0C4-4326-A1FE-F6106B7122CB}">
   <dimension ref="A6:F31"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.6640625" customWidth="1"/>
+    <col min="1" max="1" width="17.7109375" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
-    <col min="3" max="3" width="15.6640625" customWidth="1"/>
-    <col min="4" max="5" width="16.33203125" customWidth="1"/>
-    <col min="6" max="6" width="18.44140625" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="5" width="16.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="14" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="12" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14"/>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="14" t="s">
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12"/>
+      <c r="E6" s="12"/>
+      <c r="F6" s="12"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="12" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14"/>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C8" s="17"/>
-      <c r="D8" s="17"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B7" s="12"/>
+      <c r="C7" s="12"/>
+      <c r="D7" s="12"/>
+      <c r="E7" s="12"/>
+      <c r="F7" s="12"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="15" t="s">
+      <c r="C9" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="D9" s="13"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="16"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C10" s="14"/>
+      <c r="D10" s="14"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
-      <c r="F11" s="15"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="15"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C13" s="14"/>
+      <c r="D13" s="14"/>
+      <c r="E13" s="14"/>
+      <c r="F13" s="14"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="16"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C14" s="14"/>
+      <c r="D14" s="14"/>
+      <c r="E14" s="14"/>
+      <c r="F14" s="14"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="16"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C15" s="14"/>
+      <c r="D15" s="14"/>
+      <c r="E15" s="14"/>
+      <c r="F15" s="14"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-    </row>
-    <row r="18" spans="1:6" ht="30.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="18" t="s">
+      <c r="C16" s="14"/>
+      <c r="D16" s="14"/>
+      <c r="E16" s="14"/>
+      <c r="F16" s="14"/>
+    </row>
+    <row r="18" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="A18" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="19"/>
+      <c r="B18" s="17"/>
       <c r="C18" s="3" t="s">
         <v>13</v>
       </c>
@@ -1499,129 +1498,129 @@
         <v>16</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="13" t="s">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="13"/>
+      <c r="B19" s="11"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="13" t="s">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="13"/>
+      <c r="B20" s="11"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="13" t="s">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="13"/>
+      <c r="B21" s="11"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="13" t="s">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="13"/>
+      <c r="B22" s="11"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="13" t="s">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="13"/>
+      <c r="B23" s="11"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="13" t="s">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="13"/>
+      <c r="B24" s="11"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="13" t="s">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="11"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="13" t="s">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="13"/>
+      <c r="B26" s="11"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="13" t="s">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="13"/>
+      <c r="B27" s="11"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="13" t="s">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="13"/>
+      <c r="B28" s="11"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="13" t="s">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="13"/>
+      <c r="B29" s="11"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="13" t="s">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="13"/>
+      <c r="B30" s="11"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="11"/>
-      <c r="B31" s="12"/>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" s="18"/>
+      <c r="B31" s="19"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
@@ -1629,6 +1628,18 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:F7"/>
@@ -1642,18 +1653,6 @@
     <mergeCell ref="C16:F16"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -1663,30 +1662,30 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48CC2D19-F3C5-43A0-9FF0-0B76506917B4}">
   <dimension ref="B1:H7"/>
-  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="3.44140625" customWidth="1"/>
-    <col min="2" max="2" width="5.5546875" customWidth="1"/>
-    <col min="3" max="3" width="13.33203125" customWidth="1"/>
-    <col min="4" max="4" width="18.5546875" customWidth="1"/>
-    <col min="5" max="5" width="19.33203125" customWidth="1"/>
-    <col min="6" max="6" width="12.44140625" customWidth="1"/>
-    <col min="7" max="7" width="19.88671875" customWidth="1"/>
-    <col min="8" max="8" width="21.109375" customWidth="1"/>
+    <col min="1" max="1" width="3.42578125" customWidth="1"/>
+    <col min="2" max="2" width="5.5703125" customWidth="1"/>
+    <col min="3" max="3" width="13.28515625" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" customWidth="1"/>
+    <col min="5" max="5" width="19.28515625" customWidth="1"/>
+    <col min="6" max="6" width="12.42578125" customWidth="1"/>
+    <col min="7" max="7" width="19.85546875" customWidth="1"/>
+    <col min="8" max="8" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="2:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B1" s="23"/>
       <c r="C1" s="24"/>
       <c r="D1" s="29" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="E1" s="30"/>
       <c r="F1" s="30"/>
       <c r="G1" s="31"/>
       <c r="H1" s="32"/>
     </row>
-    <row r="2" spans="2:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="2:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="25"/>
       <c r="C2" s="26"/>
       <c r="D2" s="35" t="s">
@@ -1701,7 +1700,7 @@
       </c>
       <c r="H2" s="33"/>
     </row>
-    <row r="3" spans="2:8" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="2:8" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B3" s="27"/>
       <c r="C3" s="28"/>
       <c r="D3" s="35" t="s">
@@ -1716,8 +1715,8 @@
       </c>
       <c r="H3" s="34"/>
     </row>
-    <row r="4" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
-    <row r="5" spans="2:8" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="5" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="20" t="s">
         <v>34</v>
       </c>
@@ -1725,7 +1724,7 @@
       <c r="D5" s="21"/>
       <c r="E5" s="22"/>
     </row>
-    <row r="7" spans="2:8" ht="42.6" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:8" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">
         <v>35</v>
       </c>
@@ -1736,16 +1735,16 @@
         <v>37</v>
       </c>
       <c r="E7" s="8" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="F7" s="8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G7" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>38</v>
-      </c>
-      <c r="H7" s="9" t="s">
-        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cambio: Formato de consumo de agua actualizado
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/ConsumoAgua/FORMATO REPORTE DE CONSUMO DE AGUA.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/ConsumoAgua/FORMATO REPORTE DE CONSUMO DE AGUA.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Segunda Etapa\ConsumoAgua\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\ConsumoAgua\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Rediseño\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\ConsumoAgua\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C18F562-758A-45ED-9E8A-483A196678AC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EC8645C-53CD-44C7-B48E-3B45DAD2B788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{AFFB72D5-6F10-40F3-BC87-67601F9B819B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{AFFB72D5-6F10-40F3-BC87-67601F9B819B}"/>
   </bookViews>
   <sheets>
-    <sheet name="REPORTE MENSUAL" sheetId="1" r:id="rId1"/>
-    <sheet name="REPORTE CONSUMO DIARIO" sheetId="2" r:id="rId2"/>
+    <sheet name="REPORTE MENSUAL" sheetId="5" r:id="rId1"/>
+    <sheet name="REPORTE ACUMULADO" sheetId="1" r:id="rId2"/>
+    <sheet name="REPORTE CONSUMO DIARIO" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029" calcOnSave="0" concurrentCalc="0"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="45">
   <si>
     <t>FORMATO: 6A</t>
   </si>
@@ -285,12 +286,66 @@
   <si>
     <t>Volumen de Agua Bombeado (m3)</t>
   </si>
+  <si>
+    <r>
+      <t>Caudal 
+(m</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/s)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Volumen de agua captado 
+(m</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -350,6 +405,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="6">
     <fill>
@@ -582,10 +644,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -615,33 +679,36 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -694,8 +761,10 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{BCA61926-BA31-4F31-A4E0-3D9FC820986E}"/>
+    <cellStyle name="Normal 3" xfId="2" xr:uid="{0C33E97E-AE17-47CA-B235-42C0F323BCC8}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -711,6 +780,111 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>440487</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>157155</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Imagen1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5462C4D3-CE76-4CC3-9356-F05C5777602B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="285750" y="342900"/>
+          <a:ext cx="1335837" cy="766755"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>285750</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>152400</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>438806</xdr:colOff>
+      <xdr:row>5</xdr:row>
+      <xdr:rowOff>157155</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="5" name="Imagen1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE5EFBE7-6E99-4036-83B2-3A2CD80A72F4}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="285750" y="342900"/>
+          <a:ext cx="1334156" cy="766755"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -924,7 +1098,7 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
@@ -1347,6 +1521,181 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DFA4058-9522-4FE3-936B-1B70EA4B700B}">
+  <dimension ref="A6:G18"/>
+  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="17.7109375" customWidth="1"/>
+    <col min="2" max="2" width="15" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" customWidth="1"/>
+    <col min="4" max="5" width="16.28515625" customWidth="1"/>
+    <col min="6" max="6" width="18.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="13" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>4</v>
+      </c>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+    </row>
+    <row r="18" spans="1:7" ht="62.25" x14ac:dyDescent="0.25">
+      <c r="A18" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="B18" s="20"/>
+      <c r="C18" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="20"/>
+      <c r="E18" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="F18" s="20"/>
+      <c r="G18" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="14">
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="C18:D18"/>
+    <mergeCell ref="E18:F18"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C11:F11"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51A04389-D0C4-4326-A1FE-F6106B7122CB}">
   <dimension ref="A6:F31"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1359,28 +1708,28 @@
   </cols>
   <sheetData>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="12"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="12"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C8" s="15"/>
-      <c r="D8" s="15"/>
+      <c r="C8" s="14"/>
+      <c r="D8" s="14"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -1389,12 +1738,12 @@
       <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="13"/>
-      <c r="E9" s="13"/>
-      <c r="F9" s="13"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="12"/>
+      <c r="F9" s="12"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -1403,10 +1752,10 @@
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="14"/>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
+      <c r="C10" s="15"/>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -1415,10 +1764,10 @@
       <c r="B11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="13"/>
-      <c r="D11" s="13"/>
-      <c r="E11" s="13"/>
-      <c r="F11" s="13"/>
+      <c r="C11" s="12"/>
+      <c r="D11" s="12"/>
+      <c r="E11" s="12"/>
+      <c r="F11" s="12"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -1427,10 +1776,10 @@
       <c r="B12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="13"/>
-      <c r="D12" s="13"/>
-      <c r="E12" s="13"/>
-      <c r="F12" s="13"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="12"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -1439,10 +1788,10 @@
       <c r="B13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="14"/>
-      <c r="D13" s="14"/>
-      <c r="E13" s="14"/>
-      <c r="F13" s="14"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15"/>
+      <c r="F13" s="15"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -1451,10 +1800,10 @@
       <c r="B14" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="14"/>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
+      <c r="C14" s="15"/>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -1463,10 +1812,10 @@
       <c r="B15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -1475,16 +1824,16 @@
       <c r="B16" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
     </row>
     <row r="18" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="19" t="s">
         <v>12</v>
       </c>
-      <c r="B18" s="17"/>
+      <c r="B18" s="20"/>
       <c r="C18" s="3" t="s">
         <v>13</v>
       </c>
@@ -1499,128 +1848,128 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="11" t="s">
+      <c r="A19" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="11"/>
+      <c r="B19" s="18"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="11" t="s">
+      <c r="A20" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="11"/>
+      <c r="B20" s="18"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="11" t="s">
+      <c r="A21" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="11"/>
+      <c r="B21" s="18"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="11" t="s">
+      <c r="A22" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="11"/>
+      <c r="B22" s="18"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="11" t="s">
+      <c r="A23" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="11"/>
+      <c r="B23" s="18"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="11" t="s">
+      <c r="A24" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="11"/>
+      <c r="B24" s="18"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="11" t="s">
+      <c r="A25" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="11"/>
+      <c r="B25" s="18"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="11" t="s">
+      <c r="A26" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="11"/>
+      <c r="B26" s="18"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="11" t="s">
+      <c r="A27" s="18" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="11"/>
+      <c r="B27" s="18"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="11" t="s">
+      <c r="A28" s="18" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="11"/>
+      <c r="B28" s="18"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="11" t="s">
+      <c r="A29" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="11"/>
+      <c r="B29" s="18"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="11" t="s">
+      <c r="A30" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="11"/>
+      <c r="B30" s="18"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="18"/>
-      <c r="B31" s="19"/>
+      <c r="A31" s="16"/>
+      <c r="B31" s="17"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
@@ -1628,18 +1977,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:F7"/>
@@ -1653,13 +1990,25 @@
     <mergeCell ref="C16:F16"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48CC2D19-F3C5-43A0-9FF0-0B76506917B4}">
   <dimension ref="B1:H7"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -1675,54 +2024,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="23"/>
-      <c r="C1" s="24"/>
-      <c r="D1" s="29" t="s">
+      <c r="B1" s="24"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="30" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="30"/>
-      <c r="F1" s="30"/>
-      <c r="G1" s="31"/>
-      <c r="H1" s="32"/>
+      <c r="E1" s="31"/>
+      <c r="F1" s="31"/>
+      <c r="G1" s="32"/>
+      <c r="H1" s="33"/>
     </row>
     <row r="2" spans="2:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25"/>
-      <c r="C2" s="26"/>
-      <c r="D2" s="35" t="s">
+      <c r="B2" s="26"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="36"/>
+      <c r="E2" s="37"/>
       <c r="F2" s="4" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="33"/>
+      <c r="H2" s="34"/>
     </row>
     <row r="3" spans="2:8" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="27"/>
-      <c r="C3" s="28"/>
-      <c r="D3" s="35" t="s">
+      <c r="B3" s="28"/>
+      <c r="C3" s="29"/>
+      <c r="D3" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="36"/>
+      <c r="E3" s="37"/>
       <c r="F3" s="5" t="s">
         <v>33</v>
       </c>
       <c r="G3" s="6">
         <v>44136</v>
       </c>
-      <c r="H3" s="34"/>
+      <c r="H3" s="35"/>
     </row>
     <row r="4" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="21" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="21"/>
-      <c r="E5" s="22"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="22"/>
+      <c r="E5" s="23"/>
     </row>
     <row r="7" spans="2:8" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">

</xml_diff>

<commit_message>
Nuevo formato reporte consumo agua
</commit_message>
<xml_diff>
--- a/GestionAmbiental/wwwroot/ExcelTemplates/ConsumoAgua/FORMATO REPORTE DE CONSUMO DE AGUA.xlsx
+++ b/GestionAmbiental/wwwroot/ExcelTemplates/ConsumoAgua/FORMATO REPORTE DE CONSUMO DE AGUA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24701"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Electrodata\Marcobre\Rediseño\Marcobre-GestionAmbiental\GestionAmbiental\wwwroot\ExcelTemplates\ConsumoAgua\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9EC8645C-53CD-44C7-B48E-3B45DAD2B788}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04C9AB27-B8FE-4C8B-A30E-242DD216C30B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{AFFB72D5-6F10-40F3-BC87-67601F9B819B}"/>
+    <workbookView xWindow="2940" yWindow="1920" windowWidth="28800" windowHeight="15435" xr2:uid="{AFFB72D5-6F10-40F3-BC87-67601F9B819B}"/>
   </bookViews>
   <sheets>
     <sheet name="REPORTE MENSUAL" sheetId="5" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="73" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="57">
   <si>
     <t>FORMATO: 6A</t>
   </si>
@@ -339,6 +339,42 @@
       </rPr>
       <t>)</t>
     </r>
+  </si>
+  <si>
+    <t>DIRECCIÓN DE ADMINISTRACIÓN EN RECURSOS HÍDRICOS</t>
+  </si>
+  <si>
+    <t>FORMATO 6</t>
+  </si>
+  <si>
+    <t>Unidad Operativa</t>
+  </si>
+  <si>
+    <t>Mina Justa</t>
+  </si>
+  <si>
+    <t>Tipo / N° Resolución</t>
+  </si>
+  <si>
+    <t>REPORTE DE VOLÚMENES DE AGUA CAPTADOS POR LOS USUARIOS CON SISTEMA PROPIO DE ABASTECIMIENTO DE AGUA</t>
+  </si>
+  <si>
+    <t>Nombre de Usuario</t>
+  </si>
+  <si>
+    <t>Código de Usuario</t>
+  </si>
+  <si>
+    <t>(1)</t>
+  </si>
+  <si>
+    <t>(2)</t>
+  </si>
+  <si>
+    <t>(3)</t>
+  </si>
+  <si>
+    <t>(4)</t>
   </si>
 </sst>
 </file>
@@ -445,7 +481,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="17">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -643,13 +679,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -683,31 +728,49 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -784,26 +847,26 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
+      <xdr:colOff>1131796</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>89647</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>440487</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>157155</xdr:rowOff>
+      <xdr:colOff>918526</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>181537</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Imagen1">
+        <xdr:cNvPr id="7" name="Imagen1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5462C4D3-CE76-4CC3-9356-F05C5777602B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4E78E671-675D-43B1-9B67-661D3E6CE223}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
+        <xdr:cNvPicPr preferRelativeResize="0">
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
@@ -821,58 +884,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="285750" y="342900"/>
-          <a:ext cx="1335837" cy="766755"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>285750</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>152400</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>438806</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>157155</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Imagen1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FE5EFBE7-6E99-4036-83B2-3A2CD80A72F4}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="285750" y="342900"/>
-          <a:ext cx="1334156" cy="766755"/>
+          <a:off x="1131796" y="89647"/>
+          <a:ext cx="1131436" cy="663390"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1522,141 +1535,163 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2DFA4058-9522-4FE3-936B-1B70EA4B700B}">
-  <dimension ref="A6:G18"/>
+  <dimension ref="A5:H18"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="17.7109375" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="15.7109375" customWidth="1"/>
     <col min="4" max="5" width="16.28515625" customWidth="1"/>
     <col min="6" max="6" width="18.42578125" customWidth="1"/>
   </cols>
   <sheetData>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+    </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
-      <c r="G6" s="13"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
-      <c r="G7" s="13"/>
+      <c r="A6" s="17"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
+      <c r="G6" s="17"/>
+    </row>
+    <row r="7" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="18" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="18"/>
+      <c r="C7" s="18"/>
+      <c r="D7" s="18"/>
+      <c r="E7" s="18"/>
+      <c r="F7" s="18"/>
+      <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
+      <c r="G8" t="s">
+        <v>46</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B9" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="B9" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B10" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="11" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="C11" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+    </row>
+    <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B12" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B14" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="B14" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B15" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B15" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B16" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-    </row>
-    <row r="18" spans="1:7" ht="62.25" x14ac:dyDescent="0.25">
+      <c r="A16" s="1"/>
+      <c r="B16" s="11"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>53</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="D17" s="16"/>
+      <c r="E17" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="14" t="s">
+        <v>56</v>
+      </c>
+      <c r="H17" s="13"/>
+    </row>
+    <row r="18" spans="1:8" ht="62.25" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
         <v>36</v>
       </c>
@@ -1674,7 +1709,10 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="14">
+  <mergeCells count="17">
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="E17:F17"/>
     <mergeCell ref="A6:G6"/>
     <mergeCell ref="A7:G7"/>
     <mergeCell ref="C18:D18"/>
@@ -1691,6 +1729,9 @@
     <mergeCell ref="C11:F11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A17:G17" numberStoredAsText="1"/>
+  </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -1708,28 +1749,28 @@
   </cols>
   <sheetData>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="D6" s="13"/>
-      <c r="E6" s="13"/>
-      <c r="F6" s="13"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
+      <c r="D6" s="17"/>
+      <c r="E6" s="17"/>
+      <c r="F6" s="17"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="17" t="s">
         <v>1</v>
       </c>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-      <c r="E7" s="13"/>
-      <c r="F7" s="13"/>
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="17"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
+      <c r="C8" s="23"/>
+      <c r="D8" s="23"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -1738,12 +1779,12 @@
       <c r="B9" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="21" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="12"/>
+      <c r="D9" s="21"/>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
@@ -1752,10 +1793,10 @@
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
@@ -1764,10 +1805,10 @@
       <c r="B11" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="12"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
@@ -1776,10 +1817,10 @@
       <c r="B12" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
+      <c r="C12" s="21"/>
+      <c r="D12" s="21"/>
+      <c r="E12" s="21"/>
+      <c r="F12" s="21"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
@@ -1788,10 +1829,10 @@
       <c r="B13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="15"/>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
+      <c r="C13" s="22"/>
+      <c r="D13" s="22"/>
+      <c r="E13" s="22"/>
+      <c r="F13" s="22"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
@@ -1800,10 +1841,10 @@
       <c r="B14" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+      <c r="C14" s="22"/>
+      <c r="D14" s="22"/>
+      <c r="E14" s="22"/>
+      <c r="F14" s="22"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
@@ -1812,10 +1853,10 @@
       <c r="B15" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
+      <c r="C15" s="22"/>
+      <c r="D15" s="22"/>
+      <c r="E15" s="22"/>
+      <c r="F15" s="22"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
@@ -1824,10 +1865,10 @@
       <c r="B16" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
+      <c r="C16" s="22"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
     </row>
     <row r="18" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A18" s="19" t="s">
@@ -1848,128 +1889,128 @@
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" s="18" t="s">
+      <c r="A19" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="18"/>
+      <c r="B19" s="24"/>
       <c r="C19" s="10"/>
       <c r="D19" s="10"/>
       <c r="E19" s="10"/>
       <c r="F19" s="10"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" s="18" t="s">
+      <c r="A20" s="24" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="18"/>
+      <c r="B20" s="24"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" s="18" t="s">
+      <c r="A21" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="18"/>
+      <c r="B21" s="24"/>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" s="18" t="s">
+      <c r="A22" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="18"/>
+      <c r="B22" s="24"/>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="10"/>
       <c r="F22" s="10"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" s="18" t="s">
+      <c r="A23" s="24" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="18"/>
+      <c r="B23" s="24"/>
       <c r="C23" s="10"/>
       <c r="D23" s="10"/>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
+      <c r="A24" s="24" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="18"/>
+      <c r="B24" s="24"/>
       <c r="C24" s="10"/>
       <c r="D24" s="10"/>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" s="18" t="s">
+      <c r="A25" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="18"/>
+      <c r="B25" s="24"/>
       <c r="C25" s="10"/>
       <c r="D25" s="10"/>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" s="18" t="s">
+      <c r="A26" s="24" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="18"/>
+      <c r="B26" s="24"/>
       <c r="C26" s="10"/>
       <c r="D26" s="10"/>
       <c r="E26" s="10"/>
       <c r="F26" s="10"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" s="18" t="s">
+      <c r="A27" s="24" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="18"/>
+      <c r="B27" s="24"/>
       <c r="C27" s="10"/>
       <c r="D27" s="10"/>
       <c r="E27" s="10"/>
       <c r="F27" s="10"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="18" t="s">
+      <c r="A28" s="24" t="s">
         <v>26</v>
       </c>
-      <c r="B28" s="18"/>
+      <c r="B28" s="24"/>
       <c r="C28" s="10"/>
       <c r="D28" s="10"/>
       <c r="E28" s="10"/>
       <c r="F28" s="10"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" s="18" t="s">
+      <c r="A29" s="24" t="s">
         <v>27</v>
       </c>
-      <c r="B29" s="18"/>
+      <c r="B29" s="24"/>
       <c r="C29" s="10"/>
       <c r="D29" s="10"/>
       <c r="E29" s="10"/>
       <c r="F29" s="10"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" s="18" t="s">
+      <c r="A30" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="18"/>
+      <c r="B30" s="24"/>
       <c r="C30" s="10"/>
       <c r="D30" s="10"/>
       <c r="E30" s="10"/>
       <c r="F30" s="10"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="16"/>
-      <c r="B31" s="17"/>
+      <c r="A31" s="25"/>
+      <c r="B31" s="26"/>
       <c r="C31" s="10"/>
       <c r="D31" s="10"/>
       <c r="E31" s="10"/>
@@ -1977,6 +2018,18 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A6:F6"/>
     <mergeCell ref="A7:F7"/>
@@ -1990,18 +2043,6 @@
     <mergeCell ref="C16:F16"/>
     <mergeCell ref="C15:F15"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A31:B31"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A30:B30"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2024,54 +2065,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="24"/>
-      <c r="C1" s="25"/>
-      <c r="D1" s="30" t="s">
+      <c r="B1" s="30"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="E1" s="31"/>
-      <c r="F1" s="31"/>
-      <c r="G1" s="32"/>
-      <c r="H1" s="33"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="37"/>
+      <c r="G1" s="38"/>
+      <c r="H1" s="39"/>
     </row>
     <row r="2" spans="2:8" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="26"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="36" t="s">
+      <c r="B2" s="32"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="42" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="37"/>
+      <c r="E2" s="43"/>
       <c r="F2" s="4" t="s">
         <v>30</v>
       </c>
       <c r="G2" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="H2" s="34"/>
+      <c r="H2" s="40"/>
     </row>
     <row r="3" spans="2:8" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="28"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="36" t="s">
+      <c r="B3" s="34"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="42" t="s">
         <v>32</v>
       </c>
-      <c r="E3" s="37"/>
+      <c r="E3" s="43"/>
       <c r="F3" s="5" t="s">
         <v>33</v>
       </c>
       <c r="G3" s="6">
         <v>44136</v>
       </c>
-      <c r="H3" s="35"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="21" t="s">
+      <c r="B5" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="21"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="23"/>
+      <c r="C5" s="27"/>
+      <c r="D5" s="28"/>
+      <c r="E5" s="29"/>
     </row>
     <row r="7" spans="2:8" ht="40.5" x14ac:dyDescent="0.25">
       <c r="B7" s="8" t="s">

</xml_diff>